<commit_message>
docs: embed live screenshots into individual WTN-A06 report Word docx
</commit_message>
<xml_diff>
--- a/backend/api_list_snapshot.xlsx
+++ b/backend/api_list_snapshot.xlsx
@@ -1235,7 +1235,7 @@
     <row r="23" ht="24" customHeight="1">
       <c r="A23" s="4" t="inlineStr">
         <is>
-          <t>6. System Monitoring &amp; Health Domain</t>
+          <t>7. System Monitoring &amp; Health Domain</t>
         </is>
       </c>
       <c r="B23" s="5" t="inlineStr">
@@ -1273,7 +1273,7 @@
     <row r="24" ht="24" customHeight="1">
       <c r="A24" s="4" t="inlineStr">
         <is>
-          <t>6. System Monitoring &amp; Health Domain</t>
+          <t>7. System Monitoring &amp; Health Domain</t>
         </is>
       </c>
       <c r="B24" s="5" t="inlineStr">

</xml_diff>

<commit_message>
WTN-A07: Complete Trainer Worker implementation with Redis scheduled queue and MinIO
</commit_message>
<xml_diff>
--- a/backend/api_list_snapshot.xlsx
+++ b/backend/api_list_snapshot.xlsx
@@ -499,7 +499,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G25"/>
+  <dimension ref="A1:G27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -718,67 +718,68 @@
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
+          <t>/api/v1/datasets/import-huggingface</t>
+        </is>
+      </c>
+      <c r="C9" s="6" t="inlineStr">
+        <is>
+          <t>POST</t>
+        </is>
+      </c>
+      <c r="D9" s="5" t="inlineStr">
+        <is>
+          <t>Import Hugging Face Dataset</t>
+        </is>
+      </c>
+      <c r="E9" s="5" t="inlineStr">
+        <is>
+          <t>Download Token Classification / NER dataset from Hugging Face and store in MinIO bucket 'datasets'</t>
+        </is>
+      </c>
+      <c r="F9" s="5" t="inlineStr">
+        <is>
+          <t>dataset_name (query, string, Optional)
+split (query, string, Optional)</t>
+        </is>
+      </c>
+      <c r="G9" s="4" t="inlineStr">
+        <is>
+          <t>201, 422</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="24" customHeight="1">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>2. Dataset Management Domain</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
           <t>/api/v1/datasets</t>
         </is>
       </c>
-      <c r="C9" s="7" t="inlineStr">
+      <c r="C10" s="7" t="inlineStr">
         <is>
           <t>GET</t>
         </is>
       </c>
-      <c r="D9" s="5" t="inlineStr">
+      <c r="D10" s="5" t="inlineStr">
         <is>
           <t>List Datasets</t>
         </is>
       </c>
-      <c r="E9" s="5" t="inlineStr">
+      <c r="E10" s="5" t="inlineStr">
         <is>
           <t>List datasets with pagination.</t>
         </is>
       </c>
-      <c r="F9" s="5" t="inlineStr">
+      <c r="F10" s="5" t="inlineStr">
         <is>
           <t>skip (query, integer, Optional)
 limit (query, integer, Optional)</t>
         </is>
       </c>
-      <c r="G9" s="4" t="inlineStr">
-        <is>
-          <t>200, 422</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="24" customHeight="1">
-      <c r="A10" s="4" t="inlineStr">
-        <is>
-          <t>2. Dataset Management Domain</t>
-        </is>
-      </c>
-      <c r="B10" s="5" t="inlineStr">
-        <is>
-          <t>/api/v1/datasets/{dataset_id}</t>
-        </is>
-      </c>
-      <c r="C10" s="7" t="inlineStr">
-        <is>
-          <t>GET</t>
-        </is>
-      </c>
-      <c r="D10" s="5" t="inlineStr">
-        <is>
-          <t>Get Dataset</t>
-        </is>
-      </c>
-      <c r="E10" s="5" t="inlineStr">
-        <is>
-          <t>Retrieve details for a specific dataset.</t>
-        </is>
-      </c>
-      <c r="F10" s="5" t="inlineStr">
-        <is>
-          <t>dataset_id (path, integer, Required)</t>
-        </is>
-      </c>
       <c r="G10" s="4" t="inlineStr">
         <is>
           <t>200, 422</t>
@@ -788,37 +789,37 @@
     <row r="11" ht="24" customHeight="1">
       <c r="A11" s="4" t="inlineStr">
         <is>
-          <t>3. Model Registry Domain</t>
+          <t>2. Dataset Management Domain</t>
         </is>
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>/api/v1/models/upload</t>
-        </is>
-      </c>
-      <c r="C11" s="6" t="inlineStr">
-        <is>
-          <t>POST</t>
+          <t>/api/v1/datasets/{dataset_id}</t>
+        </is>
+      </c>
+      <c r="C11" s="7" t="inlineStr">
+        <is>
+          <t>GET</t>
         </is>
       </c>
       <c r="D11" s="5" t="inlineStr">
         <is>
-          <t>Upload Model</t>
+          <t>Get Dataset</t>
         </is>
       </c>
       <c r="E11" s="5" t="inlineStr">
         <is>
-          <t>Register a new model version (Append-Only Immutability Policy).</t>
+          <t>Retrieve details for a specific dataset.</t>
         </is>
       </c>
       <c r="F11" s="5" t="inlineStr">
         <is>
-          <t>request_body (application/json)</t>
+          <t>dataset_id (path, integer, Required)</t>
         </is>
       </c>
       <c r="G11" s="4" t="inlineStr">
         <is>
-          <t>201, 422</t>
+          <t>200, 422</t>
         </is>
       </c>
     </row>
@@ -830,32 +831,32 @@
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>/api/v1/models</t>
-        </is>
-      </c>
-      <c r="C12" s="7" t="inlineStr">
-        <is>
-          <t>GET</t>
+          <t>/api/v1/models/upload</t>
+        </is>
+      </c>
+      <c r="C12" s="6" t="inlineStr">
+        <is>
+          <t>POST</t>
         </is>
       </c>
       <c r="D12" s="5" t="inlineStr">
         <is>
-          <t>List Models</t>
+          <t>Upload Model</t>
         </is>
       </c>
       <c r="E12" s="5" t="inlineStr">
         <is>
-          <t>Get audit history of all model versions.</t>
+          <t>Register a new model version (Append-Only Immutability Policy).</t>
         </is>
       </c>
       <c r="F12" s="5" t="inlineStr">
         <is>
-          <t>model_name (query, string, Optional)</t>
+          <t>request_body (application/json)</t>
         </is>
       </c>
       <c r="G12" s="4" t="inlineStr">
         <is>
-          <t>200, 422</t>
+          <t>201, 422</t>
         </is>
       </c>
     </row>
@@ -867,7 +868,7 @@
       </c>
       <c r="B13" s="5" t="inlineStr">
         <is>
-          <t>/api/v1/models/latest</t>
+          <t>/api/v1/models</t>
         </is>
       </c>
       <c r="C13" s="7" t="inlineStr">
@@ -877,12 +878,12 @@
       </c>
       <c r="D13" s="5" t="inlineStr">
         <is>
-          <t>Get Latest Model</t>
+          <t>List Models</t>
         </is>
       </c>
       <c r="E13" s="5" t="inlineStr">
         <is>
-          <t>Get latest stable model version for inference.</t>
+          <t>Get audit history of all model versions.</t>
         </is>
       </c>
       <c r="F13" s="5" t="inlineStr">
@@ -904,7 +905,7 @@
       </c>
       <c r="B14" s="5" t="inlineStr">
         <is>
-          <t>/api/v1/models/{model_id}</t>
+          <t>/api/v1/models/latest</t>
         </is>
       </c>
       <c r="C14" s="7" t="inlineStr">
@@ -914,17 +915,17 @@
       </c>
       <c r="D14" s="5" t="inlineStr">
         <is>
-          <t>Get Model By Id</t>
+          <t>Get Latest Model</t>
         </is>
       </c>
       <c r="E14" s="5" t="inlineStr">
         <is>
-          <t>Get specific model record by ID.</t>
+          <t>Get latest stable model version for inference.</t>
         </is>
       </c>
       <c r="F14" s="5" t="inlineStr">
         <is>
-          <t>model_id (path, integer, Required)</t>
+          <t>model_name (query, string, Optional)</t>
         </is>
       </c>
       <c r="G14" s="4" t="inlineStr">
@@ -936,75 +937,75 @@
     <row r="15" ht="24" customHeight="1">
       <c r="A15" s="4" t="inlineStr">
         <is>
+          <t>3. Model Registry Domain</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="inlineStr">
+        <is>
+          <t>/api/v1/models/{model_id}</t>
+        </is>
+      </c>
+      <c r="C15" s="7" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="D15" s="5" t="inlineStr">
+        <is>
+          <t>Get Model By Id</t>
+        </is>
+      </c>
+      <c r="E15" s="5" t="inlineStr">
+        <is>
+          <t>Get specific model record by ID.</t>
+        </is>
+      </c>
+      <c r="F15" s="5" t="inlineStr">
+        <is>
+          <t>model_id (path, integer, Required)</t>
+        </is>
+      </c>
+      <c r="G15" s="4" t="inlineStr">
+        <is>
+          <t>200, 422</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="24" customHeight="1">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
           <t>4. Automated Async Training Domain</t>
         </is>
       </c>
-      <c r="B15" s="5" t="inlineStr">
+      <c r="B16" s="5" t="inlineStr">
         <is>
           <t>/api/v1/training/start</t>
         </is>
       </c>
-      <c r="C15" s="6" t="inlineStr">
+      <c r="C16" s="6" t="inlineStr">
         <is>
           <t>POST</t>
         </is>
       </c>
-      <c r="D15" s="5" t="inlineStr">
+      <c r="D16" s="5" t="inlineStr">
         <is>
           <t>Start Training</t>
         </is>
       </c>
-      <c r="E15" s="5" t="inlineStr">
+      <c r="E16" s="5" t="inlineStr">
         <is>
           <t>Start heavy AI model training job asynchronously.
 Returns HTTP 202 Accepted immediately with job_id. Task pushed to Redis Queue.</t>
         </is>
       </c>
-      <c r="F15" s="5" t="inlineStr">
+      <c r="F16" s="5" t="inlineStr">
         <is>
           <t>request_body (application/json)</t>
         </is>
       </c>
-      <c r="G15" s="4" t="inlineStr">
+      <c r="G16" s="4" t="inlineStr">
         <is>
           <t>202, 422</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="24" customHeight="1">
-      <c r="A16" s="4" t="inlineStr">
-        <is>
-          <t>4. Automated Async Training Domain</t>
-        </is>
-      </c>
-      <c r="B16" s="5" t="inlineStr">
-        <is>
-          <t>/api/v1/training/status/{job_id}</t>
-        </is>
-      </c>
-      <c r="C16" s="7" t="inlineStr">
-        <is>
-          <t>GET</t>
-        </is>
-      </c>
-      <c r="D16" s="5" t="inlineStr">
-        <is>
-          <t>Get Training Status</t>
-        </is>
-      </c>
-      <c r="E16" s="5" t="inlineStr">
-        <is>
-          <t>Poll training progress and job execution status.</t>
-        </is>
-      </c>
-      <c r="F16" s="5" t="inlineStr">
-        <is>
-          <t>job_id (path, string, Required)</t>
-        </is>
-      </c>
-      <c r="G16" s="4" t="inlineStr">
-        <is>
-          <t>200, 422</t>
         </is>
       </c>
     </row>
@@ -1016,7 +1017,7 @@
       </c>
       <c r="B17" s="5" t="inlineStr">
         <is>
-          <t>/api/v1/training/cancel/{job_id}</t>
+          <t>/api/v1/training/enqueue</t>
         </is>
       </c>
       <c r="C17" s="6" t="inlineStr">
@@ -1026,54 +1027,54 @@
       </c>
       <c r="D17" s="5" t="inlineStr">
         <is>
-          <t>Cancel Training</t>
+          <t>Enqueue Scheduled Training Task</t>
         </is>
       </c>
       <c r="E17" s="5" t="inlineStr">
         <is>
-          <t>Cancel a queued training job.</t>
+          <t>Enqueue training task into Redis Sorted Set scheduled queue with a execution time delay</t>
         </is>
       </c>
       <c r="F17" s="5" t="inlineStr">
         <is>
-          <t>job_id (path, string, Required)</t>
+          <t>request_body (application/json)</t>
         </is>
       </c>
       <c r="G17" s="4" t="inlineStr">
         <is>
-          <t>200, 422</t>
+          <t>202, 422</t>
         </is>
       </c>
     </row>
     <row r="18" ht="24" customHeight="1">
       <c r="A18" s="4" t="inlineStr">
         <is>
-          <t>5. Inference Domain</t>
+          <t>4. Automated Async Training Domain</t>
         </is>
       </c>
       <c r="B18" s="5" t="inlineStr">
         <is>
-          <t>/api/v1/predict</t>
-        </is>
-      </c>
-      <c r="C18" s="6" t="inlineStr">
-        <is>
-          <t>POST</t>
+          <t>/api/v1/training/status/{job_id}</t>
+        </is>
+      </c>
+      <c r="C18" s="7" t="inlineStr">
+        <is>
+          <t>GET</t>
         </is>
       </c>
       <c r="D18" s="5" t="inlineStr">
         <is>
-          <t>Predict Inference</t>
+          <t>Get Training Status</t>
         </is>
       </c>
       <c r="E18" s="5" t="inlineStr">
         <is>
-          <t>Execute low-latency AI inference prediction.</t>
+          <t>Poll training progress and job execution status.</t>
         </is>
       </c>
       <c r="F18" s="5" t="inlineStr">
         <is>
-          <t>request_body (application/json)</t>
+          <t>job_id (path, string, Required)</t>
         </is>
       </c>
       <c r="G18" s="4" t="inlineStr">
@@ -1085,49 +1086,49 @@
     <row r="19" ht="24" customHeight="1">
       <c r="A19" s="4" t="inlineStr">
         <is>
-          <t>6. Label Studio Component Domain</t>
+          <t>4. Automated Async Training Domain</t>
         </is>
       </c>
       <c r="B19" s="5" t="inlineStr">
         <is>
-          <t>/api/v1/ls/projects</t>
-        </is>
-      </c>
-      <c r="C19" s="7" t="inlineStr">
-        <is>
-          <t>GET</t>
+          <t>/api/v1/training/cancel/{job_id}</t>
+        </is>
+      </c>
+      <c r="C19" s="6" t="inlineStr">
+        <is>
+          <t>POST</t>
         </is>
       </c>
       <c r="D19" s="5" t="inlineStr">
         <is>
-          <t>List Label Studio Projects</t>
+          <t>Cancel Training</t>
         </is>
       </c>
       <c r="E19" s="5" t="inlineStr">
         <is>
-          <t>Fetch data annotation projects from Label Studio SDK</t>
+          <t>Cancel a queued training job.</t>
         </is>
       </c>
       <c r="F19" s="5" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>job_id (path, string, Required)</t>
         </is>
       </c>
       <c r="G19" s="4" t="inlineStr">
         <is>
-          <t>200</t>
+          <t>200, 422</t>
         </is>
       </c>
     </row>
     <row r="20" ht="24" customHeight="1">
       <c r="A20" s="4" t="inlineStr">
         <is>
-          <t>6. Label Studio Component Domain</t>
+          <t>5. Inference Domain</t>
         </is>
       </c>
       <c r="B20" s="5" t="inlineStr">
         <is>
-          <t>/api/v1/ls/projects</t>
+          <t>/api/v1/predict</t>
         </is>
       </c>
       <c r="C20" s="6" t="inlineStr">
@@ -1137,12 +1138,12 @@
       </c>
       <c r="D20" s="5" t="inlineStr">
         <is>
-          <t>Create Annotation Project</t>
+          <t>Predict Inference</t>
         </is>
       </c>
       <c r="E20" s="5" t="inlineStr">
         <is>
-          <t>Create a new Label Studio data labeling project</t>
+          <t>Execute low-latency AI inference prediction.</t>
         </is>
       </c>
       <c r="F20" s="5" t="inlineStr">
@@ -1152,7 +1153,7 @@
       </c>
       <c r="G20" s="4" t="inlineStr">
         <is>
-          <t>201, 422</t>
+          <t>200, 422</t>
         </is>
       </c>
     </row>
@@ -1164,177 +1165,251 @@
       </c>
       <c r="B21" s="5" t="inlineStr">
         <is>
+          <t>/api/v1/ls/projects</t>
+        </is>
+      </c>
+      <c r="C21" s="7" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="D21" s="5" t="inlineStr">
+        <is>
+          <t>List Label Studio Projects</t>
+        </is>
+      </c>
+      <c r="E21" s="5" t="inlineStr">
+        <is>
+          <t>Fetch data annotation projects from Label Studio SDK</t>
+        </is>
+      </c>
+      <c r="F21" s="5" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="G21" s="4" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="24" customHeight="1">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>6. Label Studio Component Domain</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="inlineStr">
+        <is>
+          <t>/api/v1/ls/projects</t>
+        </is>
+      </c>
+      <c r="C22" s="6" t="inlineStr">
+        <is>
+          <t>POST</t>
+        </is>
+      </c>
+      <c r="D22" s="5" t="inlineStr">
+        <is>
+          <t>Create Annotation Project</t>
+        </is>
+      </c>
+      <c r="E22" s="5" t="inlineStr">
+        <is>
+          <t>Create a new Label Studio data labeling project</t>
+        </is>
+      </c>
+      <c r="F22" s="5" t="inlineStr">
+        <is>
+          <t>request_body (application/json)</t>
+        </is>
+      </c>
+      <c r="G22" s="4" t="inlineStr">
+        <is>
+          <t>201, 422</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="24" customHeight="1">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>6. Label Studio Component Domain</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="inlineStr">
+        <is>
           <t>/api/v1/ls/tasks/import</t>
         </is>
       </c>
-      <c r="C21" s="6" t="inlineStr">
+      <c r="C23" s="6" t="inlineStr">
         <is>
           <t>POST</t>
         </is>
       </c>
-      <c r="D21" s="5" t="inlineStr">
+      <c r="D23" s="5" t="inlineStr">
         <is>
           <t>Import Dataset Tasks</t>
         </is>
       </c>
-      <c r="E21" s="5" t="inlineStr">
+      <c r="E23" s="5" t="inlineStr">
         <is>
           <t>Import raw dataset files/links into Label Studio project for labeling</t>
         </is>
       </c>
-      <c r="F21" s="5" t="inlineStr">
+      <c r="F23" s="5" t="inlineStr">
         <is>
           <t>project_id (query, integer, Required)
 request_body (application/json)</t>
         </is>
       </c>
-      <c r="G21" s="4" t="inlineStr">
+      <c r="G23" s="4" t="inlineStr">
         <is>
           <t>200, 422</t>
         </is>
       </c>
     </row>
-    <row r="22" ht="24" customHeight="1">
-      <c r="A22" s="4" t="inlineStr">
+    <row r="24" ht="24" customHeight="1">
+      <c r="A24" s="4" t="inlineStr">
         <is>
           <t>6. Label Studio Component Domain</t>
         </is>
       </c>
-      <c r="B22" s="5" t="inlineStr">
+      <c r="B24" s="5" t="inlineStr">
         <is>
           <t>/api/v1/ls/annotations/export</t>
         </is>
       </c>
-      <c r="C22" s="7" t="inlineStr">
+      <c r="C24" s="7" t="inlineStr">
         <is>
           <t>GET</t>
         </is>
       </c>
-      <c r="D22" s="5" t="inlineStr">
+      <c r="D24" s="5" t="inlineStr">
         <is>
           <t>Export Labeled Annotations</t>
         </is>
       </c>
-      <c r="E22" s="5" t="inlineStr">
+      <c r="E24" s="5" t="inlineStr">
         <is>
           <t>Export completed data annotations from Label Studio to PostgreSQL/MinIO</t>
         </is>
       </c>
-      <c r="F22" s="5" t="inlineStr">
+      <c r="F24" s="5" t="inlineStr">
         <is>
           <t>project_id (query, integer, Required)
 export_format (query, string, Optional)</t>
         </is>
       </c>
-      <c r="G22" s="4" t="inlineStr">
+      <c r="G24" s="4" t="inlineStr">
         <is>
           <t>200, 422</t>
         </is>
       </c>
     </row>
-    <row r="23" ht="24" customHeight="1">
-      <c r="A23" s="4" t="inlineStr">
+    <row r="25" ht="24" customHeight="1">
+      <c r="A25" s="4" t="inlineStr">
         <is>
           <t>7. System Monitoring &amp; Health Domain</t>
         </is>
       </c>
-      <c r="B23" s="5" t="inlineStr">
+      <c r="B25" s="5" t="inlineStr">
         <is>
           <t>/api/v1/system/health</t>
         </is>
       </c>
-      <c r="C23" s="7" t="inlineStr">
+      <c r="C25" s="7" t="inlineStr">
         <is>
           <t>GET</t>
         </is>
       </c>
-      <c r="D23" s="5" t="inlineStr">
+      <c r="D25" s="5" t="inlineStr">
         <is>
           <t>System Health Check</t>
         </is>
       </c>
-      <c r="E23" s="5" t="inlineStr">
+      <c r="E25" s="5" t="inlineStr">
         <is>
           <t>System Health Check endpoint for Container Orchestration (Docker/Kubernetes).
 PING test for PostgreSQL, MinIO, and Redis. Returns 200 OK or 503 Service Unavailable.</t>
         </is>
       </c>
-      <c r="F23" s="5" t="inlineStr">
+      <c r="F25" s="5" t="inlineStr">
         <is>
           <t>None</t>
         </is>
       </c>
-      <c r="G23" s="4" t="inlineStr">
+      <c r="G25" s="4" t="inlineStr">
         <is>
           <t>200</t>
         </is>
       </c>
     </row>
-    <row r="24" ht="24" customHeight="1">
-      <c r="A24" s="4" t="inlineStr">
+    <row r="26" ht="24" customHeight="1">
+      <c r="A26" s="4" t="inlineStr">
         <is>
           <t>7. System Monitoring &amp; Health Domain</t>
         </is>
       </c>
-      <c r="B24" s="5" t="inlineStr">
+      <c r="B26" s="5" t="inlineStr">
         <is>
           <t>/api/v1/system/logs</t>
         </is>
       </c>
-      <c r="C24" s="7" t="inlineStr">
+      <c r="C26" s="7" t="inlineStr">
         <is>
           <t>GET</t>
         </is>
       </c>
-      <c r="D24" s="5" t="inlineStr">
+      <c r="D26" s="5" t="inlineStr">
         <is>
           <t>Get System Logs</t>
         </is>
       </c>
-      <c r="E24" s="5" t="inlineStr">
+      <c r="E26" s="5" t="inlineStr">
         <is>
           <t>Retrieve machine-readable Structured JSON Logs.</t>
         </is>
       </c>
-      <c r="F24" s="5" t="inlineStr">
+      <c r="F26" s="5" t="inlineStr">
         <is>
           <t>None</t>
         </is>
       </c>
-      <c r="G24" s="4" t="inlineStr">
+      <c r="G26" s="4" t="inlineStr">
         <is>
           <t>200</t>
         </is>
       </c>
     </row>
-    <row r="25" ht="24" customHeight="1">
-      <c r="A25" s="4" t="inlineStr">
+    <row r="27" ht="24" customHeight="1">
+      <c r="A27" s="4" t="inlineStr">
         <is>
           <t>7. System Monitoring &amp; Health Domain</t>
         </is>
       </c>
-      <c r="B25" s="5" t="inlineStr">
+      <c r="B27" s="5" t="inlineStr">
         <is>
           <t>/</t>
         </is>
       </c>
-      <c r="C25" s="7" t="inlineStr">
+      <c r="C27" s="7" t="inlineStr">
         <is>
           <t>GET</t>
         </is>
       </c>
-      <c r="D25" s="5" t="inlineStr">
+      <c r="D27" s="5" t="inlineStr">
         <is>
           <t>Root Health Status</t>
         </is>
       </c>
-      <c r="E25" s="5" t="inlineStr"/>
-      <c r="F25" s="5" t="inlineStr">
+      <c r="E27" s="5" t="inlineStr"/>
+      <c r="F27" s="5" t="inlineStr">
         <is>
           <t>None</t>
         </is>
       </c>
-      <c r="G25" s="4" t="inlineStr">
+      <c r="G27" s="4" t="inlineStr">
         <is>
           <t>200</t>
         </is>

</xml_diff>